<commit_message>
feat(ancillaries): add OmanAir supplier and runs, update AirSMCairo rules and SeatMap sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/platform_core_data/supplier-features/ancillaries/shared/ancillaries-baseline/test_design/TestCases_AncillariesSeatMap.xlsx
+++ b/platform_core_data/supplier-features/ancillaries/shared/ancillaries-baseline/test_design/TestCases_AncillariesSeatMap.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,7 +14,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$P$80</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -31,46 +30,57 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
-      <color rgb="00808080"/>
+      <name val="Calibri"/>
+      <color rgb="FF808080"/>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="14"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <i val="1"/>
       <color rgb="FF9E9E9E"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF9E9E9E"/>
       <sz val="9"/>
@@ -82,17 +92,20 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <i val="1"/>
       <color rgb="FF9E9E9E"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF9E9E9E"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="9"/>
     </font>
     <font>
@@ -100,6 +113,7 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -112,42 +126,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
+        <fgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
+        <fgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
+        <fgColor rgb="FFC6E0B4"/>
       </patternFill>
     </fill>
   </fills>
@@ -161,17 +175,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -280,7 +295,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -663,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S127"/>
+  <dimension ref="A1:S125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -682,12 +697,10 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="17" max="19"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
+    <row r="1" ht="33.95" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No.</t>
@@ -841,17 +854,17 @@
           <t>The wizard used to have 3 steps. It changed to 2 steps on 15 Sep 2026.</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
       <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr"/>
+      <c r="R2" s="4" t="n"/>
       <c r="S2" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -910,18 +923,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="n"/>
       <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr"/>
+      <c r="R3" s="4" t="n"/>
       <c r="S3" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -980,18 +993,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="4" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
       <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R4" s="4" t="inlineStr"/>
+      <c r="R4" s="4" t="n"/>
       <c r="S4" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1049,22 +1062,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
           <t>The map was rebuilt on 15 Sep 2026. It is now [role="dialog"] labelled by #seat-map-shell-title, with body.seat-map-shell-open. Old scripts looking for a PrimeNG p-dialog will fail.</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
       <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr"/>
+      <c r="R5" s="4" t="n"/>
       <c r="S5" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1123,18 +1136,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="3" t="n"/>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr"/>
+      <c r="R6" s="4" t="n"/>
       <c r="S6" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1193,18 +1206,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="4" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr"/>
-      <c r="O7" s="4" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr"/>
+      <c r="R7" s="4" t="n"/>
       <c r="S7" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1273,16 +1286,16 @@
           <t>Classes: seat--free, seat--unavailable, seat--not-offered, seat--female, seat--selected-other. A seat that costs money has none of --free or --unavailable; read its price from aria-label.</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr"/>
-      <c r="N8" s="4" t="inlineStr"/>
-      <c r="O8" s="4" t="inlineStr"/>
-      <c r="P8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="n"/>
       <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr"/>
+      <c r="R8" s="4" t="n"/>
       <c r="S8" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1339,22 +1352,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="n"/>
       <c r="L9" s="3" t="inlineStr">
         <is>
           <t>Read from aria-label on each seat button.</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr"/>
-      <c r="N9" s="4" t="inlineStr"/>
-      <c r="O9" s="4" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
       <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R9" s="4" t="inlineStr"/>
+      <c r="R9" s="4" t="n"/>
       <c r="S9" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1413,18 +1426,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr"/>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="3" t="n"/>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="n"/>
       <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R10" s="4" t="inlineStr"/>
+      <c r="R10" s="4" t="n"/>
       <c r="S10" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1481,18 +1494,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="4" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr"/>
-      <c r="O11" s="4" t="inlineStr"/>
-      <c r="P11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="3" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="n"/>
+      <c r="O11" s="4" t="n"/>
+      <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R11" s="4" t="inlineStr"/>
+      <c r="R11" s="4" t="n"/>
       <c r="S11" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1555,17 +1568,17 @@
           <t>You need a second flight on a different aircraft type; which aircraft flies a route is decided by the airline, so this cannot always be arranged.</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="n"/>
+      <c r="O12" s="4" t="n"/>
+      <c r="P12" s="4" t="n"/>
       <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R12" s="4" t="inlineStr"/>
+      <c r="R12" s="4" t="n"/>
       <c r="S12" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1624,18 +1637,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr"/>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="3" t="n"/>
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4" t="n"/>
+      <c r="O13" s="4" t="n"/>
+      <c r="P13" s="4" t="n"/>
       <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R13" s="4" t="inlineStr"/>
+      <c r="R13" s="4" t="n"/>
       <c r="S13" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1694,18 +1707,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="3" t="n"/>
+      <c r="M14" s="4" t="n"/>
+      <c r="N14" s="4" t="n"/>
+      <c r="O14" s="4" t="n"/>
+      <c r="P14" s="4" t="n"/>
       <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr"/>
+      <c r="R14" s="4" t="n"/>
       <c r="S14" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1769,17 +1782,17 @@
           <t>'Chargeable seat' was missing from the 15 Sep map but present again on 17 Sep - it depends on the flight, so its absence is not a fault.</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr"/>
-      <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr"/>
+      <c r="L15" s="3" t="n"/>
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4" t="n"/>
+      <c r="O15" s="4" t="n"/>
+      <c r="P15" s="4" t="n"/>
       <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R15" s="4" t="inlineStr"/>
+      <c r="R15" s="4" t="n"/>
       <c r="S15" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1838,18 +1851,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="3" t="n"/>
+      <c r="M16" s="4" t="n"/>
+      <c r="N16" s="4" t="n"/>
+      <c r="O16" s="4" t="n"/>
+      <c r="P16" s="4" t="n"/>
       <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R16" s="4" t="inlineStr"/>
+      <c r="R16" s="4" t="n"/>
       <c r="S16" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1908,18 +1921,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr"/>
-      <c r="O17" s="4" t="inlineStr"/>
-      <c r="P17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="n"/>
+      <c r="L17" s="3" t="n"/>
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4" t="n"/>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4" t="n"/>
       <c r="Q17" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R17" s="4" t="inlineStr"/>
+      <c r="R17" s="4" t="n"/>
       <c r="S17" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1988,10 +2001,10 @@
           <t>Classes: seat--female (always), plus seat--unavailable and seat--not-offered only when the passenger is male.</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
+      <c r="M18" s="4" t="n"/>
+      <c r="N18" s="4" t="n"/>
+      <c r="O18" s="4" t="n"/>
+      <c r="P18" s="4" t="n"/>
       <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -2061,18 +2074,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr"/>
-      <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr"/>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4" t="n"/>
+      <c r="O19" s="4" t="n"/>
+      <c r="P19" s="4" t="n"/>
       <c r="Q19" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R19" s="4" t="inlineStr"/>
+      <c r="R19" s="4" t="n"/>
       <c r="S19" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2131,18 +2144,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
-      <c r="O20" s="4" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="3" t="n"/>
+      <c r="M20" s="4" t="n"/>
+      <c r="N20" s="4" t="n"/>
+      <c r="O20" s="4" t="n"/>
+      <c r="P20" s="4" t="n"/>
       <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R20" s="4" t="inlineStr"/>
+      <c r="R20" s="4" t="n"/>
       <c r="S20" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2200,18 +2213,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr"/>
-      <c r="M21" s="4" t="inlineStr"/>
-      <c r="N21" s="4" t="inlineStr"/>
-      <c r="O21" s="4" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="3" t="n"/>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="n"/>
+      <c r="O21" s="4" t="n"/>
+      <c r="P21" s="4" t="n"/>
       <c r="Q21" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R21" s="4" t="inlineStr"/>
+      <c r="R21" s="4" t="n"/>
       <c r="S21" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2282,16 +2295,16 @@
           <t>Buttons: button.confirm-action and button.confirm-reset.</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr"/>
-      <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="n"/>
+      <c r="N22" s="4" t="n"/>
+      <c r="O22" s="4" t="n"/>
+      <c r="P22" s="4" t="n"/>
       <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R22" s="4" t="inlineStr"/>
+      <c r="R22" s="4" t="n"/>
       <c r="S22" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2349,18 +2362,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr"/>
-      <c r="M23" s="4" t="inlineStr"/>
-      <c r="N23" s="4" t="inlineStr"/>
-      <c r="O23" s="4" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="3" t="n"/>
+      <c r="M23" s="4" t="n"/>
+      <c r="N23" s="4" t="n"/>
+      <c r="O23" s="4" t="n"/>
+      <c r="P23" s="4" t="n"/>
       <c r="Q23" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R23" s="4" t="inlineStr"/>
+      <c r="R23" s="4" t="n"/>
       <c r="S23" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2417,18 +2430,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr"/>
-      <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr"/>
-      <c r="O24" s="4" t="inlineStr"/>
-      <c r="P24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="n"/>
+      <c r="L24" s="3" t="n"/>
+      <c r="M24" s="4" t="n"/>
+      <c r="N24" s="4" t="n"/>
+      <c r="O24" s="4" t="n"/>
+      <c r="P24" s="4" t="n"/>
       <c r="Q24" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R24" s="4" t="inlineStr"/>
+      <c r="R24" s="4" t="n"/>
       <c r="S24" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2489,18 +2502,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="4" t="inlineStr"/>
-      <c r="O25" s="4" t="inlineStr"/>
-      <c r="P25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="n"/>
+      <c r="L25" s="3" t="n"/>
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4" t="n"/>
+      <c r="O25" s="4" t="n"/>
+      <c r="P25" s="4" t="n"/>
       <c r="Q25" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R25" s="4" t="inlineStr"/>
+      <c r="R25" s="4" t="n"/>
       <c r="S25" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2557,18 +2570,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
-      <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="n"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="n"/>
+      <c r="O26" s="4" t="n"/>
+      <c r="P26" s="4" t="n"/>
       <c r="Q26" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R26" s="4" t="inlineStr"/>
+      <c r="R26" s="4" t="n"/>
       <c r="S26" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2636,16 +2649,16 @@
           <t>Class: seat--selected-other.</t>
         </is>
       </c>
-      <c r="M27" s="4" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr"/>
-      <c r="O27" s="4" t="inlineStr"/>
-      <c r="P27" s="4" t="inlineStr"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="n"/>
+      <c r="O27" s="4" t="n"/>
+      <c r="P27" s="4" t="n"/>
       <c r="Q27" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R27" s="4" t="inlineStr"/>
+      <c r="R27" s="4" t="n"/>
       <c r="S27" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2704,18 +2717,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
-      <c r="O28" s="4" t="inlineStr"/>
-      <c r="P28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="n"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="4" t="n"/>
+      <c r="N28" s="4" t="n"/>
+      <c r="O28" s="4" t="n"/>
+      <c r="P28" s="4" t="n"/>
       <c r="Q28" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R28" s="4" t="inlineStr"/>
+      <c r="R28" s="4" t="n"/>
       <c r="S28" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2783,16 +2796,16 @@
           <t>Class: seat--selected-other.</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr"/>
-      <c r="O29" s="4" t="inlineStr"/>
-      <c r="P29" s="4" t="inlineStr"/>
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4" t="n"/>
+      <c r="O29" s="4" t="n"/>
+      <c r="P29" s="4" t="n"/>
       <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R29" s="4" t="inlineStr"/>
+      <c r="R29" s="4" t="n"/>
       <c r="S29" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2851,18 +2864,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr"/>
-      <c r="O30" s="4" t="inlineStr"/>
-      <c r="P30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="4" t="n"/>
+      <c r="N30" s="4" t="n"/>
+      <c r="O30" s="4" t="n"/>
+      <c r="P30" s="4" t="n"/>
       <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R30" s="4" t="inlineStr"/>
+      <c r="R30" s="4" t="n"/>
       <c r="S30" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2920,18 +2933,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr"/>
-      <c r="O31" s="4" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="n"/>
+      <c r="L31" s="3" t="n"/>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4" t="n"/>
+      <c r="O31" s="4" t="n"/>
+      <c r="P31" s="4" t="n"/>
       <c r="Q31" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R31" s="4" t="inlineStr"/>
+      <c r="R31" s="4" t="n"/>
       <c r="S31" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2990,18 +3003,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="4" t="inlineStr"/>
-      <c r="N32" s="4" t="inlineStr"/>
-      <c r="O32" s="4" t="inlineStr"/>
-      <c r="P32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="n"/>
+      <c r="L32" s="3" t="n"/>
+      <c r="M32" s="4" t="n"/>
+      <c r="N32" s="4" t="n"/>
+      <c r="O32" s="4" t="n"/>
+      <c r="P32" s="4" t="n"/>
       <c r="Q32" s="4" t="inlineStr">
         <is>
           <t>Bundle + Seat</t>
         </is>
       </c>
-      <c r="R32" s="4" t="inlineStr"/>
+      <c r="R32" s="4" t="n"/>
       <c r="S32" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3069,7 +3082,7 @@
 27 Sep 2026 (run-006): reproduced on flynas KSA, XY584. Confirmed as a bug by the business.</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr"/>
+      <c r="L33" s="3" t="n"/>
       <c r="M33" s="4" t="inlineStr">
         <is>
           <t>Under 'Plus', all 36 seats marked 'Chargeable seat' showed 'available for Free' (e.g. 5A); the total did not change. Under 'Value' they were priced correctly.</t>
@@ -3095,7 +3108,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R33" s="4" t="inlineStr"/>
+      <c r="R33" s="4" t="n"/>
       <c r="S33" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3160,17 +3173,17 @@
           <t>Was impossible to test before 15 Sep 2026, because no paid seat had ever been seen.</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="4" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr"/>
-      <c r="O34" s="4" t="inlineStr"/>
-      <c r="P34" s="4" t="inlineStr"/>
+      <c r="L34" s="3" t="n"/>
+      <c r="M34" s="4" t="n"/>
+      <c r="N34" s="4" t="n"/>
+      <c r="O34" s="4" t="n"/>
+      <c r="P34" s="4" t="n"/>
       <c r="Q34" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R34" s="4" t="inlineStr"/>
+      <c r="R34" s="4" t="n"/>
       <c r="S34" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3234,17 +3247,17 @@
           <t>Seen on 15 Sep: Free / 422.91 / 1,097.91. Seen on 17 Sep: section Y-1 'from EGP 642', section Y-2 'Free - EGP 642'.</t>
         </is>
       </c>
-      <c r="L35" s="3" t="inlineStr"/>
-      <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr"/>
-      <c r="O35" s="4" t="inlineStr"/>
-      <c r="P35" s="4" t="inlineStr"/>
+      <c r="L35" s="3" t="n"/>
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4" t="n"/>
+      <c r="O35" s="4" t="n"/>
+      <c r="P35" s="4" t="n"/>
       <c r="Q35" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R35" s="4" t="inlineStr"/>
+      <c r="R35" s="4" t="n"/>
       <c r="S35" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3309,17 +3322,17 @@
           <t>Checked on 15 Sep 2026: 1,800 + 1,295.82 = 3,095.82, total 10,413.82 EGP.</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr"/>
-      <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr"/>
-      <c r="O36" s="4" t="inlineStr"/>
-      <c r="P36" s="4" t="inlineStr"/>
+      <c r="L36" s="3" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="n"/>
+      <c r="O36" s="4" t="n"/>
+      <c r="P36" s="4" t="n"/>
       <c r="Q36" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R36" s="4" t="inlineStr"/>
+      <c r="R36" s="4" t="n"/>
       <c r="S36" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3386,7 +3399,7 @@
 27 Sep 2026 (run-006): business confirms this is a feature, not a defect - bundle change clears ancillaries, it does not recalculate them. Not retried; the stuck-wizard observation from the earlier 16 attempts stands as a separate item.</t>
         </is>
       </c>
-      <c r="L37" s="3" t="inlineStr"/>
+      <c r="L37" s="3" t="n"/>
       <c r="M37" s="4" t="inlineStr">
         <is>
           <t>The case's own premise was wrong. Per business decision, changing the fare package is not meant to recalculate the seats - it clears the ancillaries (seats, meals, bags) so the agent re-selects them under the new bundle. This run's attempts to observe a downgrade never reached that point: after downgrading Plus -&gt; Value, advancing to step 2 failed twice with a sold-out ssr-quote error and the wizard stayed on step 1 with no visible message - a separate, still-open observation (tied to V6-12), not a failure of this case.</t>
@@ -3412,7 +3425,7 @@
           <t>Bundle + Seat</t>
         </is>
       </c>
-      <c r="R37" s="4" t="inlineStr"/>
+      <c r="R37" s="4" t="n"/>
       <c r="S37" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3469,18 +3482,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr"/>
-      <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr"/>
-      <c r="O38" s="4" t="inlineStr"/>
-      <c r="P38" s="4" t="inlineStr"/>
+      <c r="K38" s="4" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="n"/>
+      <c r="O38" s="4" t="n"/>
+      <c r="P38" s="4" t="n"/>
       <c r="Q38" s="4" t="inlineStr">
         <is>
           <t>Bundle</t>
         </is>
       </c>
-      <c r="R38" s="4" t="inlineStr"/>
+      <c r="R38" s="4" t="n"/>
       <c r="S38" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3545,17 +3558,17 @@
           <t>This test used to record the fault. Since 15 Sep 2026 it guards against the fault returning.</t>
         </is>
       </c>
-      <c r="L39" s="3" t="inlineStr"/>
-      <c r="M39" s="4" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr"/>
-      <c r="O39" s="4" t="inlineStr"/>
-      <c r="P39" s="4" t="inlineStr"/>
+      <c r="L39" s="3" t="n"/>
+      <c r="M39" s="4" t="n"/>
+      <c r="N39" s="4" t="n"/>
+      <c r="O39" s="4" t="n"/>
+      <c r="P39" s="4" t="n"/>
       <c r="Q39" s="4" t="inlineStr">
         <is>
           <t>Bundle</t>
         </is>
       </c>
-      <c r="R39" s="4" t="inlineStr"/>
+      <c r="R39" s="4" t="n"/>
       <c r="S39" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3614,18 +3627,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" s="4" t="inlineStr"/>
-      <c r="O40" s="4" t="inlineStr"/>
-      <c r="P40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="n"/>
+      <c r="L40" s="3" t="n"/>
+      <c r="M40" s="4" t="n"/>
+      <c r="N40" s="4" t="n"/>
+      <c r="O40" s="4" t="n"/>
+      <c r="P40" s="4" t="n"/>
       <c r="Q40" s="4" t="inlineStr">
         <is>
           <t>Bundle + Seat</t>
         </is>
       </c>
-      <c r="R40" s="4" t="inlineStr"/>
+      <c r="R40" s="4" t="n"/>
       <c r="S40" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3684,12 +3697,12 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="3" t="inlineStr"/>
-      <c r="M41" s="4" t="inlineStr"/>
-      <c r="N41" s="4" t="inlineStr"/>
-      <c r="O41" s="4" t="inlineStr"/>
-      <c r="P41" s="4" t="inlineStr"/>
+      <c r="K41" s="4" t="n"/>
+      <c r="L41" s="3" t="n"/>
+      <c r="M41" s="4" t="n"/>
+      <c r="N41" s="4" t="n"/>
+      <c r="O41" s="4" t="n"/>
+      <c r="P41" s="4" t="n"/>
       <c r="Q41" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -3764,11 +3777,11 @@
           <t>Confirmed on 15 Sep 2026.</t>
         </is>
       </c>
-      <c r="L42" s="3" t="inlineStr"/>
-      <c r="M42" s="4" t="inlineStr"/>
-      <c r="N42" s="4" t="inlineStr"/>
-      <c r="O42" s="4" t="inlineStr"/>
-      <c r="P42" s="4" t="inlineStr"/>
+      <c r="L42" s="3" t="n"/>
+      <c r="M42" s="4" t="n"/>
+      <c r="N42" s="4" t="n"/>
+      <c r="O42" s="4" t="n"/>
+      <c r="P42" s="4" t="n"/>
       <c r="Q42" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -3848,10 +3861,10 @@
           <t>data-seat-id is base64. Decoded: &lt;flightKey&gt;#&lt;seat&gt;#&lt;overallState&gt;#&lt;perPaxStates&gt;#&lt;attributes&gt;#&lt;cabin&gt;, where perPaxStates is like 0:Blocked,1:AvailablePaid.</t>
         </is>
       </c>
-      <c r="M43" s="4" t="inlineStr"/>
-      <c r="N43" s="4" t="inlineStr"/>
-      <c r="O43" s="4" t="inlineStr"/>
-      <c r="P43" s="4" t="inlineStr"/>
+      <c r="M43" s="4" t="n"/>
+      <c r="N43" s="4" t="n"/>
+      <c r="O43" s="4" t="n"/>
+      <c r="P43" s="4" t="n"/>
       <c r="Q43" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -3919,18 +3932,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr"/>
-      <c r="M44" s="4" t="inlineStr"/>
-      <c r="N44" s="4" t="inlineStr"/>
-      <c r="O44" s="4" t="inlineStr"/>
-      <c r="P44" s="4" t="inlineStr"/>
+      <c r="K44" s="4" t="n"/>
+      <c r="L44" s="3" t="n"/>
+      <c r="M44" s="4" t="n"/>
+      <c r="N44" s="4" t="n"/>
+      <c r="O44" s="4" t="n"/>
+      <c r="P44" s="4" t="n"/>
       <c r="Q44" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R44" s="4" t="inlineStr"/>
+      <c r="R44" s="4" t="n"/>
       <c r="S44" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -3994,11 +4007,11 @@
           <t>Confirmed on 15 Sep 2026.</t>
         </is>
       </c>
-      <c r="L45" s="3" t="inlineStr"/>
-      <c r="M45" s="4" t="inlineStr"/>
-      <c r="N45" s="4" t="inlineStr"/>
-      <c r="O45" s="4" t="inlineStr"/>
-      <c r="P45" s="4" t="inlineStr"/>
+      <c r="L45" s="3" t="n"/>
+      <c r="M45" s="4" t="n"/>
+      <c r="N45" s="4" t="n"/>
+      <c r="O45" s="4" t="n"/>
+      <c r="P45" s="4" t="n"/>
       <c r="Q45" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -4073,11 +4086,11 @@
           <t>CORRECTED 17 Sep 2026: it is 'Ms' OR 'Mrs', and the title list is the same for children and adults.</t>
         </is>
       </c>
-      <c r="L46" s="3" t="inlineStr"/>
-      <c r="M46" s="4" t="inlineStr"/>
-      <c r="N46" s="4" t="inlineStr"/>
-      <c r="O46" s="4" t="inlineStr"/>
-      <c r="P46" s="4" t="inlineStr"/>
+      <c r="L46" s="3" t="n"/>
+      <c r="M46" s="4" t="n"/>
+      <c r="N46" s="4" t="n"/>
+      <c r="O46" s="4" t="n"/>
+      <c r="P46" s="4" t="n"/>
       <c r="Q46" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -4145,18 +4158,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr"/>
-      <c r="M47" s="4" t="inlineStr"/>
-      <c r="N47" s="4" t="inlineStr"/>
-      <c r="O47" s="4" t="inlineStr"/>
-      <c r="P47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="n"/>
+      <c r="L47" s="3" t="n"/>
+      <c r="M47" s="4" t="n"/>
+      <c r="N47" s="4" t="n"/>
+      <c r="O47" s="4" t="n"/>
+      <c r="P47" s="4" t="n"/>
       <c r="Q47" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R47" s="4" t="inlineStr"/>
+      <c r="R47" s="4" t="n"/>
       <c r="S47" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4215,18 +4228,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr"/>
-      <c r="M48" s="4" t="inlineStr"/>
-      <c r="N48" s="4" t="inlineStr"/>
-      <c r="O48" s="4" t="inlineStr"/>
-      <c r="P48" s="4" t="inlineStr"/>
+      <c r="K48" s="4" t="n"/>
+      <c r="L48" s="3" t="n"/>
+      <c r="M48" s="4" t="n"/>
+      <c r="N48" s="4" t="n"/>
+      <c r="O48" s="4" t="n"/>
+      <c r="P48" s="4" t="n"/>
       <c r="Q48" s="4" t="inlineStr">
         <is>
           <t>Seat + Meal + Baggage</t>
         </is>
       </c>
-      <c r="R48" s="4" t="inlineStr"/>
+      <c r="R48" s="4" t="n"/>
       <c r="S48" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4292,17 +4305,17 @@
           <t>Re-run this against the 15-minute limit before go-live. Waiting for real expiry is slow, so run it as a separate scheduled check.</t>
         </is>
       </c>
-      <c r="L49" s="3" t="inlineStr"/>
-      <c r="M49" s="4" t="inlineStr"/>
-      <c r="N49" s="4" t="inlineStr"/>
-      <c r="O49" s="4" t="inlineStr"/>
-      <c r="P49" s="4" t="inlineStr"/>
+      <c r="L49" s="3" t="n"/>
+      <c r="M49" s="4" t="n"/>
+      <c r="N49" s="4" t="n"/>
+      <c r="O49" s="4" t="n"/>
+      <c r="P49" s="4" t="n"/>
       <c r="Q49" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R49" s="4" t="inlineStr"/>
+      <c r="R49" s="4" t="n"/>
       <c r="S49" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4364,17 +4377,17 @@
           <t>Never press 'Book' - it creates a real booking and takes money from the agency wallet.</t>
         </is>
       </c>
-      <c r="L50" s="3" t="inlineStr"/>
-      <c r="M50" s="4" t="inlineStr"/>
-      <c r="N50" s="4" t="inlineStr"/>
-      <c r="O50" s="4" t="inlineStr"/>
-      <c r="P50" s="4" t="inlineStr"/>
+      <c r="L50" s="3" t="n"/>
+      <c r="M50" s="4" t="n"/>
+      <c r="N50" s="4" t="n"/>
+      <c r="O50" s="4" t="n"/>
+      <c r="P50" s="4" t="n"/>
       <c r="Q50" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R50" s="4" t="inlineStr"/>
+      <c r="R50" s="4" t="n"/>
       <c r="S50" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4432,18 +4445,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K51" s="4" t="inlineStr"/>
-      <c r="L51" s="3" t="inlineStr"/>
-      <c r="M51" s="4" t="inlineStr"/>
-      <c r="N51" s="4" t="inlineStr"/>
-      <c r="O51" s="4" t="inlineStr"/>
-      <c r="P51" s="4" t="inlineStr"/>
+      <c r="K51" s="4" t="n"/>
+      <c r="L51" s="3" t="n"/>
+      <c r="M51" s="4" t="n"/>
+      <c r="N51" s="4" t="n"/>
+      <c r="O51" s="4" t="n"/>
+      <c r="P51" s="4" t="n"/>
       <c r="Q51" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R51" s="4" t="inlineStr"/>
+      <c r="R51" s="4" t="n"/>
       <c r="S51" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4508,7 +4521,7 @@
 Commented out 27 Sep 2026 (Mohanad Dawood): not to be executed.</t>
         </is>
       </c>
-      <c r="L52" s="26" t="inlineStr"/>
+      <c r="L52" s="26" t="n"/>
       <c r="M52" s="27" t="inlineStr">
         <is>
           <t>Commented out - not to be executed.</t>
@@ -4534,7 +4547,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R52" s="27" t="inlineStr"/>
+      <c r="R52" s="27" t="n"/>
       <c r="S52" s="27" t="inlineStr">
         <is>
           <t>Rejected</t>
@@ -4596,17 +4609,17 @@
           <t>The token lasts 60 minutes while testing and 15 minutes when live.</t>
         </is>
       </c>
-      <c r="L53" s="3" t="inlineStr"/>
-      <c r="M53" s="4" t="inlineStr"/>
-      <c r="N53" s="4" t="inlineStr"/>
-      <c r="O53" s="4" t="inlineStr"/>
-      <c r="P53" s="4" t="inlineStr"/>
+      <c r="L53" s="3" t="n"/>
+      <c r="M53" s="4" t="n"/>
+      <c r="N53" s="4" t="n"/>
+      <c r="O53" s="4" t="n"/>
+      <c r="P53" s="4" t="n"/>
       <c r="Q53" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R53" s="4" t="inlineStr"/>
+      <c r="R53" s="4" t="n"/>
       <c r="S53" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4670,17 +4683,17 @@
           <t>The mechanical parts can be checked automatically; whether it looks right needs a person.</t>
         </is>
       </c>
-      <c r="L54" s="3" t="inlineStr"/>
-      <c r="M54" s="4" t="inlineStr"/>
-      <c r="N54" s="4" t="inlineStr"/>
-      <c r="O54" s="4" t="inlineStr"/>
-      <c r="P54" s="4" t="inlineStr"/>
+      <c r="L54" s="3" t="n"/>
+      <c r="M54" s="4" t="n"/>
+      <c r="N54" s="4" t="n"/>
+      <c r="O54" s="4" t="n"/>
+      <c r="P54" s="4" t="n"/>
       <c r="Q54" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R54" s="4" t="inlineStr"/>
+      <c r="R54" s="4" t="n"/>
       <c r="S54" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4738,18 +4751,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K55" s="4" t="inlineStr"/>
-      <c r="L55" s="3" t="inlineStr"/>
-      <c r="M55" s="4" t="inlineStr"/>
-      <c r="N55" s="4" t="inlineStr"/>
-      <c r="O55" s="4" t="inlineStr"/>
-      <c r="P55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="n"/>
+      <c r="L55" s="3" t="n"/>
+      <c r="M55" s="4" t="n"/>
+      <c r="N55" s="4" t="n"/>
+      <c r="O55" s="4" t="n"/>
+      <c r="P55" s="4" t="n"/>
       <c r="Q55" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R55" s="4" t="inlineStr"/>
+      <c r="R55" s="4" t="n"/>
       <c r="S55" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -4814,11 +4827,11 @@
           <t>Tagged 28 Sep 2026: needs a supplier that sells a second cabin. Air Cairo sells Economy only (cards read "No Business"), so these are excluded there.</t>
         </is>
       </c>
-      <c r="L56" s="3" t="inlineStr"/>
-      <c r="M56" s="4" t="inlineStr"/>
-      <c r="N56" s="4" t="inlineStr"/>
-      <c r="O56" s="4" t="inlineStr"/>
-      <c r="P56" s="4" t="inlineStr"/>
+      <c r="L56" s="3" t="n"/>
+      <c r="M56" s="4" t="n"/>
+      <c r="N56" s="4" t="n"/>
+      <c r="O56" s="4" t="n"/>
+      <c r="P56" s="4" t="n"/>
       <c r="Q56" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -4894,11 +4907,11 @@
 Tagged 28 Sep 2026: needs a supplier that sells a second cabin. Air Cairo sells Economy only (cards read "No Business"), so these are excluded there.</t>
         </is>
       </c>
-      <c r="L57" s="3" t="inlineStr"/>
-      <c r="M57" s="4" t="inlineStr"/>
-      <c r="N57" s="4" t="inlineStr"/>
-      <c r="O57" s="4" t="inlineStr"/>
-      <c r="P57" s="4" t="inlineStr"/>
+      <c r="L57" s="3" t="n"/>
+      <c r="M57" s="4" t="n"/>
+      <c r="N57" s="4" t="n"/>
+      <c r="O57" s="4" t="n"/>
+      <c r="P57" s="4" t="n"/>
       <c r="Q57" s="4" t="inlineStr">
         <is>
           <t>Bundle + Seat</t>
@@ -4973,11 +4986,11 @@
 Tagged 28 Sep 2026: needs a supplier that sells a second cabin. Air Cairo sells Economy only (cards read "No Business"), so these are excluded there.</t>
         </is>
       </c>
-      <c r="L58" s="3" t="inlineStr"/>
-      <c r="M58" s="4" t="inlineStr"/>
-      <c r="N58" s="4" t="inlineStr"/>
-      <c r="O58" s="4" t="inlineStr"/>
-      <c r="P58" s="4" t="inlineStr"/>
+      <c r="L58" s="3" t="n"/>
+      <c r="M58" s="4" t="n"/>
+      <c r="N58" s="4" t="n"/>
+      <c r="O58" s="4" t="n"/>
+      <c r="P58" s="4" t="n"/>
       <c r="Q58" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -5050,11 +5063,11 @@
 Tagged 28 Sep 2026: needs a supplier that sells a second cabin. Air Cairo sells Economy only (cards read "No Business"), so these are excluded there.</t>
         </is>
       </c>
-      <c r="L59" s="3" t="inlineStr"/>
-      <c r="M59" s="4" t="inlineStr"/>
-      <c r="N59" s="4" t="inlineStr"/>
-      <c r="O59" s="4" t="inlineStr"/>
-      <c r="P59" s="4" t="inlineStr"/>
+      <c r="L59" s="3" t="n"/>
+      <c r="M59" s="4" t="n"/>
+      <c r="N59" s="4" t="n"/>
+      <c r="O59" s="4" t="n"/>
+      <c r="P59" s="4" t="n"/>
       <c r="Q59" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -5130,11 +5143,11 @@
 Tagged 28 Sep 2026: needs a supplier that sells a second cabin. Air Cairo sells Economy only (cards read "No Business"), so these are excluded there.</t>
         </is>
       </c>
-      <c r="L60" s="3" t="inlineStr"/>
-      <c r="M60" s="4" t="inlineStr"/>
-      <c r="N60" s="4" t="inlineStr"/>
-      <c r="O60" s="4" t="inlineStr"/>
-      <c r="P60" s="4" t="inlineStr"/>
+      <c r="L60" s="3" t="n"/>
+      <c r="M60" s="4" t="n"/>
+      <c r="N60" s="4" t="n"/>
+      <c r="O60" s="4" t="n"/>
+      <c r="P60" s="4" t="n"/>
       <c r="Q60" s="4" t="inlineStr">
         <is>
           <t>Bundle + Meal + Baggage</t>
@@ -5208,11 +5221,11 @@
 Tagged 28 Sep 2026: needs a supplier that sells a second cabin. Air Cairo sells Economy only (cards read "No Business"), so these are excluded there.</t>
         </is>
       </c>
-      <c r="L61" s="3" t="inlineStr"/>
-      <c r="M61" s="4" t="inlineStr"/>
-      <c r="N61" s="4" t="inlineStr"/>
-      <c r="O61" s="4" t="inlineStr"/>
-      <c r="P61" s="4" t="inlineStr"/>
+      <c r="L61" s="3" t="n"/>
+      <c r="M61" s="4" t="n"/>
+      <c r="N61" s="4" t="n"/>
+      <c r="O61" s="4" t="n"/>
+      <c r="P61" s="4" t="n"/>
       <c r="Q61" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
@@ -5288,17 +5301,17 @@
           <t>Checked again on 15 Sep 2026 - unchanged.</t>
         </is>
       </c>
-      <c r="L62" s="3" t="inlineStr"/>
-      <c r="M62" s="4" t="inlineStr"/>
-      <c r="N62" s="4" t="inlineStr"/>
-      <c r="O62" s="4" t="inlineStr"/>
-      <c r="P62" s="4" t="inlineStr"/>
+      <c r="L62" s="3" t="n"/>
+      <c r="M62" s="4" t="n"/>
+      <c r="N62" s="4" t="n"/>
+      <c r="O62" s="4" t="n"/>
+      <c r="P62" s="4" t="n"/>
       <c r="Q62" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R62" s="4" t="inlineStr"/>
+      <c r="R62" s="4" t="n"/>
       <c r="S62" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5356,18 +5369,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K63" s="4" t="inlineStr"/>
-      <c r="L63" s="3" t="inlineStr"/>
-      <c r="M63" s="4" t="inlineStr"/>
-      <c r="N63" s="4" t="inlineStr"/>
-      <c r="O63" s="4" t="inlineStr"/>
-      <c r="P63" s="4" t="inlineStr"/>
+      <c r="K63" s="4" t="n"/>
+      <c r="L63" s="3" t="n"/>
+      <c r="M63" s="4" t="n"/>
+      <c r="N63" s="4" t="n"/>
+      <c r="O63" s="4" t="n"/>
+      <c r="P63" s="4" t="n"/>
       <c r="Q63" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R63" s="4" t="inlineStr"/>
+      <c r="R63" s="4" t="n"/>
       <c r="S63" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5425,18 +5438,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K64" s="4" t="inlineStr"/>
-      <c r="L64" s="3" t="inlineStr"/>
-      <c r="M64" s="4" t="inlineStr"/>
-      <c r="N64" s="4" t="inlineStr"/>
-      <c r="O64" s="4" t="inlineStr"/>
-      <c r="P64" s="4" t="inlineStr"/>
+      <c r="K64" s="4" t="n"/>
+      <c r="L64" s="3" t="n"/>
+      <c r="M64" s="4" t="n"/>
+      <c r="N64" s="4" t="n"/>
+      <c r="O64" s="4" t="n"/>
+      <c r="P64" s="4" t="n"/>
       <c r="Q64" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R64" s="4" t="inlineStr"/>
+      <c r="R64" s="4" t="n"/>
       <c r="S64" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5496,18 +5509,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K65" s="4" t="inlineStr"/>
-      <c r="L65" s="3" t="inlineStr"/>
-      <c r="M65" s="4" t="inlineStr"/>
-      <c r="N65" s="4" t="inlineStr"/>
-      <c r="O65" s="4" t="inlineStr"/>
-      <c r="P65" s="4" t="inlineStr"/>
+      <c r="K65" s="4" t="n"/>
+      <c r="L65" s="3" t="n"/>
+      <c r="M65" s="4" t="n"/>
+      <c r="N65" s="4" t="n"/>
+      <c r="O65" s="4" t="n"/>
+      <c r="P65" s="4" t="n"/>
       <c r="Q65" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R65" s="4" t="inlineStr"/>
+      <c r="R65" s="4" t="n"/>
       <c r="S65" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5567,22 +5580,22 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K66" s="4" t="inlineStr"/>
+      <c r="K66" s="4" t="n"/>
       <c r="L66" s="3" t="inlineStr">
         <is>
           <t>Passengers are p-accordiontab elements inside .pax-form-accordion. A script must open a section before filling it, or the typing silently does nothing.</t>
         </is>
       </c>
-      <c r="M66" s="4" t="inlineStr"/>
-      <c r="N66" s="4" t="inlineStr"/>
-      <c r="O66" s="4" t="inlineStr"/>
-      <c r="P66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="n"/>
+      <c r="N66" s="4" t="n"/>
+      <c r="O66" s="4" t="n"/>
+      <c r="P66" s="4" t="n"/>
       <c r="Q66" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R66" s="4" t="inlineStr"/>
+      <c r="R66" s="4" t="n"/>
       <c r="S66" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5644,20 +5657,21 @@
       </c>
       <c r="K67" s="8" t="inlineStr">
         <is>
-          <t>Known behaviour, not a fault. It happens when an infant is in the party. Seen: 36,072 becoming 38,453 EGP with about 4 minutes to confirm.</t>
-        </is>
-      </c>
-      <c r="L67" s="3" t="inlineStr"/>
-      <c r="M67" s="4" t="inlineStr"/>
-      <c r="N67" s="4" t="inlineStr"/>
-      <c r="O67" s="4" t="inlineStr"/>
-      <c r="P67" s="4" t="inlineStr"/>
+          <t>Known behaviour, not a fault. It happens when an infant is in the party. Seen: 36,072 becoming 38,453 EGP with about 4 minutes to confirm.
+TESTER NOTE (30 Sep 2026, Mohanad Dawood): this price-change pop-up only happens with flynas. It does not happen with any other supplier (checked on Air Cairo, Admin, run-008), so treat this case as N/A for suppliers other than flynas.</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="n"/>
+      <c r="M67" s="4" t="n"/>
+      <c r="N67" s="4" t="n"/>
+      <c r="O67" s="4" t="n"/>
+      <c r="P67" s="4" t="n"/>
       <c r="Q67" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R67" s="4" t="inlineStr"/>
+      <c r="R67" s="4" t="n"/>
       <c r="S67" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5716,7 +5730,8 @@
       </c>
       <c r="K68" s="8" t="inlineStr">
         <is>
-          <t>Needs a price change to happen first.</t>
+          <t>Needs a price change to happen first.
+TESTER NOTE (30 Sep 2026, Mohanad Dawood): this price-change pop-up only happens with flynas. It does not happen with any other supplier (checked on Air Cairo, Admin, run-008), so treat this case as N/A for suppliers other than flynas.</t>
         </is>
       </c>
       <c r="L68" s="3" t="inlineStr">
@@ -5724,16 +5739,16 @@
           <t>The security token carries fareMismatch: true after a price change (false when there was none).</t>
         </is>
       </c>
-      <c r="M68" s="4" t="inlineStr"/>
-      <c r="N68" s="4" t="inlineStr"/>
-      <c r="O68" s="4" t="inlineStr"/>
-      <c r="P68" s="4" t="inlineStr"/>
+      <c r="M68" s="4" t="n"/>
+      <c r="N68" s="4" t="n"/>
+      <c r="O68" s="4" t="n"/>
+      <c r="P68" s="4" t="n"/>
       <c r="Q68" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R68" s="4" t="inlineStr"/>
+      <c r="R68" s="4" t="n"/>
       <c r="S68" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5792,20 +5807,21 @@
       </c>
       <c r="K69" s="8" t="inlineStr">
         <is>
-          <t>Needs a price change to happen first.</t>
-        </is>
-      </c>
-      <c r="L69" s="3" t="inlineStr"/>
-      <c r="M69" s="4" t="inlineStr"/>
-      <c r="N69" s="4" t="inlineStr"/>
-      <c r="O69" s="4" t="inlineStr"/>
-      <c r="P69" s="4" t="inlineStr"/>
+          <t>Needs a price change to happen first.
+TESTER NOTE (30 Sep 2026, Mohanad Dawood): this price-change pop-up only happens with flynas. It does not happen with any other supplier (checked on Air Cairo, Admin, run-008), so treat this case as N/A for suppliers other than flynas.</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="n"/>
+      <c r="M69" s="4" t="n"/>
+      <c r="N69" s="4" t="n"/>
+      <c r="O69" s="4" t="n"/>
+      <c r="P69" s="4" t="n"/>
       <c r="Q69" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R69" s="4" t="inlineStr"/>
+      <c r="R69" s="4" t="n"/>
       <c r="S69" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5864,20 +5880,21 @@
       </c>
       <c r="K70" s="8" t="inlineStr">
         <is>
-          <t>Needs a price change to happen first.</t>
-        </is>
-      </c>
-      <c r="L70" s="3" t="inlineStr"/>
-      <c r="M70" s="4" t="inlineStr"/>
-      <c r="N70" s="4" t="inlineStr"/>
-      <c r="O70" s="4" t="inlineStr"/>
-      <c r="P70" s="4" t="inlineStr"/>
+          <t>Needs a price change to happen first.
+TESTER NOTE (30 Sep 2026, Mohanad Dawood): this price-change pop-up only happens with flynas. It does not happen with any other supplier (checked on Air Cairo, Admin, run-008), so treat this case as N/A for suppliers other than flynas.</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="n"/>
+      <c r="M70" s="4" t="n"/>
+      <c r="N70" s="4" t="n"/>
+      <c r="O70" s="4" t="n"/>
+      <c r="P70" s="4" t="n"/>
       <c r="Q70" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R70" s="4" t="inlineStr"/>
+      <c r="R70" s="4" t="n"/>
       <c r="S70" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -5942,17 +5959,17 @@
           <t>Accepted by the business on 17 Sep 2026. It happens only sometimes and cannot be made to happen on demand.</t>
         </is>
       </c>
-      <c r="L71" s="3" t="inlineStr"/>
-      <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr"/>
-      <c r="P71" s="4" t="inlineStr"/>
+      <c r="L71" s="3" t="n"/>
+      <c r="M71" s="4" t="n"/>
+      <c r="N71" s="4" t="n"/>
+      <c r="O71" s="4" t="n"/>
+      <c r="P71" s="4" t="n"/>
       <c r="Q71" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R71" s="4" t="inlineStr"/>
+      <c r="R71" s="4" t="n"/>
       <c r="S71" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6012,18 +6029,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K72" s="4" t="inlineStr"/>
-      <c r="L72" s="3" t="inlineStr"/>
-      <c r="M72" s="4" t="inlineStr"/>
-      <c r="N72" s="4" t="inlineStr"/>
-      <c r="O72" s="4" t="inlineStr"/>
-      <c r="P72" s="4" t="inlineStr"/>
+      <c r="K72" s="4" t="n"/>
+      <c r="L72" s="3" t="n"/>
+      <c r="M72" s="4" t="n"/>
+      <c r="N72" s="4" t="n"/>
+      <c r="O72" s="4" t="n"/>
+      <c r="P72" s="4" t="n"/>
       <c r="Q72" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R72" s="4" t="inlineStr"/>
+      <c r="R72" s="4" t="n"/>
       <c r="S72" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6081,18 +6098,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K73" s="4" t="inlineStr"/>
-      <c r="L73" s="3" t="inlineStr"/>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
-      <c r="O73" s="4" t="inlineStr"/>
-      <c r="P73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="n"/>
+      <c r="L73" s="3" t="n"/>
+      <c r="M73" s="4" t="n"/>
+      <c r="N73" s="4" t="n"/>
+      <c r="O73" s="4" t="n"/>
+      <c r="P73" s="4" t="n"/>
       <c r="Q73" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R73" s="4" t="inlineStr"/>
+      <c r="R73" s="4" t="n"/>
       <c r="S73" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6149,18 +6166,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K74" s="4" t="inlineStr"/>
-      <c r="L74" s="3" t="inlineStr"/>
-      <c r="M74" s="4" t="inlineStr"/>
-      <c r="N74" s="4" t="inlineStr"/>
-      <c r="O74" s="4" t="inlineStr"/>
-      <c r="P74" s="4" t="inlineStr"/>
+      <c r="K74" s="4" t="n"/>
+      <c r="L74" s="3" t="n"/>
+      <c r="M74" s="4" t="n"/>
+      <c r="N74" s="4" t="n"/>
+      <c r="O74" s="4" t="n"/>
+      <c r="P74" s="4" t="n"/>
       <c r="Q74" s="4" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="R74" s="4" t="inlineStr"/>
+      <c r="R74" s="4" t="n"/>
       <c r="S74" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6219,18 +6236,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K75" s="4" t="inlineStr"/>
-      <c r="L75" s="3" t="inlineStr"/>
-      <c r="M75" s="4" t="inlineStr"/>
-      <c r="N75" s="4" t="inlineStr"/>
-      <c r="O75" s="4" t="inlineStr"/>
-      <c r="P75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="n"/>
+      <c r="L75" s="3" t="n"/>
+      <c r="M75" s="4" t="n"/>
+      <c r="N75" s="4" t="n"/>
+      <c r="O75" s="4" t="n"/>
+      <c r="P75" s="4" t="n"/>
       <c r="Q75" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R75" s="4" t="inlineStr"/>
+      <c r="R75" s="4" t="n"/>
       <c r="S75" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6289,18 +6306,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K76" s="4" t="inlineStr"/>
-      <c r="L76" s="3" t="inlineStr"/>
-      <c r="M76" s="4" t="inlineStr"/>
-      <c r="N76" s="4" t="inlineStr"/>
-      <c r="O76" s="4" t="inlineStr"/>
-      <c r="P76" s="4" t="inlineStr"/>
+      <c r="K76" s="4" t="n"/>
+      <c r="L76" s="3" t="n"/>
+      <c r="M76" s="4" t="n"/>
+      <c r="N76" s="4" t="n"/>
+      <c r="O76" s="4" t="n"/>
+      <c r="P76" s="4" t="n"/>
       <c r="Q76" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R76" s="4" t="inlineStr"/>
+      <c r="R76" s="4" t="n"/>
       <c r="S76" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6365,17 +6382,17 @@
           <t>Stated by the business, not yet checked in this system.</t>
         </is>
       </c>
-      <c r="L77" s="3" t="inlineStr"/>
-      <c r="M77" s="4" t="inlineStr"/>
-      <c r="N77" s="4" t="inlineStr"/>
-      <c r="O77" s="4" t="inlineStr"/>
-      <c r="P77" s="4" t="inlineStr"/>
+      <c r="L77" s="3" t="n"/>
+      <c r="M77" s="4" t="n"/>
+      <c r="N77" s="4" t="n"/>
+      <c r="O77" s="4" t="n"/>
+      <c r="P77" s="4" t="n"/>
       <c r="Q77" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R77" s="4" t="inlineStr"/>
+      <c r="R77" s="4" t="n"/>
       <c r="S77" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6433,18 +6450,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K78" s="4" t="inlineStr"/>
-      <c r="L78" s="3" t="inlineStr"/>
-      <c r="M78" s="4" t="inlineStr"/>
-      <c r="N78" s="4" t="inlineStr"/>
-      <c r="O78" s="4" t="inlineStr"/>
-      <c r="P78" s="4" t="inlineStr"/>
+      <c r="K78" s="4" t="n"/>
+      <c r="L78" s="3" t="n"/>
+      <c r="M78" s="4" t="n"/>
+      <c r="N78" s="4" t="n"/>
+      <c r="O78" s="4" t="n"/>
+      <c r="P78" s="4" t="n"/>
       <c r="Q78" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R78" s="4" t="inlineStr"/>
+      <c r="R78" s="4" t="n"/>
       <c r="S78" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6504,18 +6521,18 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K79" s="4" t="inlineStr"/>
-      <c r="L79" s="3" t="inlineStr"/>
-      <c r="M79" s="4" t="inlineStr"/>
-      <c r="N79" s="4" t="inlineStr"/>
-      <c r="O79" s="4" t="inlineStr"/>
-      <c r="P79" s="4" t="inlineStr"/>
+      <c r="K79" s="4" t="n"/>
+      <c r="L79" s="3" t="n"/>
+      <c r="M79" s="4" t="n"/>
+      <c r="N79" s="4" t="n"/>
+      <c r="O79" s="4" t="n"/>
+      <c r="P79" s="4" t="n"/>
       <c r="Q79" s="4" t="inlineStr">
         <is>
           <t>Seat</t>
         </is>
       </c>
-      <c r="R79" s="4" t="inlineStr"/>
+      <c r="R79" s="4" t="n"/>
       <c r="S79" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6580,7 +6597,7 @@
           <t>Commented out 27 Sep 2026 (Mohanad Dawood): not to be executed.</t>
         </is>
       </c>
-      <c r="L80" s="26" t="inlineStr"/>
+      <c r="L80" s="26" t="n"/>
       <c r="M80" s="27" t="inlineStr">
         <is>
           <t>Commented out - not to be executed.</t>
@@ -6606,7 +6623,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R80" s="27" t="inlineStr"/>
+      <c r="R80" s="27" t="n"/>
       <c r="S80" s="27" t="inlineStr">
         <is>
           <t>Rejected</t>
@@ -6682,7 +6699,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R81" s="4" t="inlineStr"/>
+      <c r="R81" s="4" t="n"/>
       <c r="S81" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6758,7 +6775,7 @@
           <t>Bundle + Seat</t>
         </is>
       </c>
-      <c r="R82" s="4" t="inlineStr"/>
+      <c r="R82" s="4" t="n"/>
       <c r="S82" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6834,7 +6851,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R83" s="4" t="inlineStr"/>
+      <c r="R83" s="4" t="n"/>
       <c r="S83" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6910,7 +6927,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R84" s="4" t="inlineStr"/>
+      <c r="R84" s="4" t="n"/>
       <c r="S84" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -6986,7 +7003,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R85" s="4" t="inlineStr"/>
+      <c r="R85" s="4" t="n"/>
       <c r="S85" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7062,7 +7079,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R86" s="4" t="inlineStr"/>
+      <c r="R86" s="4" t="n"/>
       <c r="S86" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7138,7 +7155,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R87" s="4" t="inlineStr"/>
+      <c r="R87" s="4" t="n"/>
       <c r="S87" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7214,7 +7231,7 @@
           <t>Baggage</t>
         </is>
       </c>
-      <c r="R88" s="4" t="inlineStr"/>
+      <c r="R88" s="4" t="n"/>
       <c r="S88" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7290,7 +7307,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R89" s="4" t="inlineStr"/>
+      <c r="R89" s="4" t="n"/>
       <c r="S89" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7367,7 +7384,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R90" s="4" t="inlineStr"/>
+      <c r="R90" s="4" t="n"/>
       <c r="S90" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7442,7 +7459,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R91" s="4" t="inlineStr"/>
+      <c r="R91" s="4" t="n"/>
       <c r="S91" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7517,7 +7534,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R92" s="4" t="inlineStr"/>
+      <c r="R92" s="4" t="n"/>
       <c r="S92" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7592,7 +7609,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R93" s="4" t="inlineStr"/>
+      <c r="R93" s="4" t="n"/>
       <c r="S93" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7685,7 +7702,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R94" s="4" t="inlineStr"/>
+      <c r="R94" s="4" t="n"/>
       <c r="S94" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7761,7 +7778,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R95" s="4" t="inlineStr"/>
+      <c r="R95" s="4" t="n"/>
       <c r="S95" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7856,7 +7873,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R96" s="4" t="inlineStr"/>
+      <c r="R96" s="4" t="n"/>
       <c r="S96" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7932,7 +7949,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R97" s="4" t="inlineStr"/>
+      <c r="R97" s="4" t="n"/>
       <c r="S97" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8025,7 +8042,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R98" s="4" t="inlineStr"/>
+      <c r="R98" s="4" t="n"/>
       <c r="S98" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8102,7 +8119,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R99" s="4" t="inlineStr"/>
+      <c r="R99" s="4" t="n"/>
       <c r="S99" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8196,7 +8213,7 @@
           <t>Baggage</t>
         </is>
       </c>
-      <c r="R100" s="4" t="inlineStr"/>
+      <c r="R100" s="4" t="n"/>
       <c r="S100" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8289,7 +8306,7 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R101" s="4" t="inlineStr"/>
+      <c r="R101" s="4" t="n"/>
       <c r="S101" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8383,7 +8400,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R102" s="4" t="inlineStr"/>
+      <c r="R102" s="4" t="n"/>
       <c r="S102" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8478,7 +8495,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R103" s="4" t="inlineStr"/>
+      <c r="R103" s="4" t="n"/>
       <c r="S103" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8571,7 +8588,7 @@
           <t>Seat</t>
         </is>
       </c>
-      <c r="R104" s="4" t="inlineStr"/>
+      <c r="R104" s="4" t="n"/>
       <c r="S104" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8643,7 +8660,7 @@
           <t>Not Seat</t>
         </is>
       </c>
-      <c r="R105" s="4" t="inlineStr"/>
+      <c r="R105" s="4" t="n"/>
       <c r="S105" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8715,7 +8732,7 @@
           <t>Meal</t>
         </is>
       </c>
-      <c r="R106" s="4" t="inlineStr"/>
+      <c r="R106" s="4" t="n"/>
       <c r="S106" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8787,7 +8804,7 @@
           <t>Meal</t>
         </is>
       </c>
-      <c r="R107" s="4" t="inlineStr"/>
+      <c r="R107" s="4" t="n"/>
       <c r="S107" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8862,7 +8879,7 @@
           <t>Meal</t>
         </is>
       </c>
-      <c r="R108" s="4" t="inlineStr"/>
+      <c r="R108" s="4" t="n"/>
       <c r="S108" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -8936,7 +8953,7 @@
           <t>Meal + Bundle</t>
         </is>
       </c>
-      <c r="R109" s="4" t="inlineStr"/>
+      <c r="R109" s="4" t="n"/>
       <c r="S109" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9009,7 +9026,7 @@
           <t>Meal</t>
         </is>
       </c>
-      <c r="R110" s="4" t="inlineStr"/>
+      <c r="R110" s="4" t="n"/>
       <c r="S110" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9080,7 +9097,7 @@
           <t>Not Meal</t>
         </is>
       </c>
-      <c r="R111" s="4" t="inlineStr"/>
+      <c r="R111" s="4" t="n"/>
       <c r="S111" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9152,7 +9169,7 @@
           <t>Baggage</t>
         </is>
       </c>
-      <c r="R112" s="4" t="inlineStr"/>
+      <c r="R112" s="4" t="n"/>
       <c r="S112" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9224,7 +9241,7 @@
           <t>Baggage</t>
         </is>
       </c>
-      <c r="R113" s="4" t="inlineStr"/>
+      <c r="R113" s="4" t="n"/>
       <c r="S113" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9297,7 +9314,7 @@
           <t>Baggage</t>
         </is>
       </c>
-      <c r="R114" s="4" t="inlineStr"/>
+      <c r="R114" s="4" t="n"/>
       <c r="S114" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9370,7 +9387,7 @@
           <t>Baggage</t>
         </is>
       </c>
-      <c r="R115" s="4" t="inlineStr"/>
+      <c r="R115" s="4" t="n"/>
       <c r="S115" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9441,7 +9458,7 @@
           <t>Not Baggage</t>
         </is>
       </c>
-      <c r="R116" s="4" t="inlineStr"/>
+      <c r="R116" s="4" t="n"/>
       <c r="S116" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9514,7 +9531,7 @@
           <t>Hold + Seat + Meal + Baggage</t>
         </is>
       </c>
-      <c r="R117" s="4" t="inlineStr"/>
+      <c r="R117" s="4" t="n"/>
       <c r="S117" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9587,7 +9604,7 @@
           <t>Hold + Pay after Hold</t>
         </is>
       </c>
-      <c r="R118" s="4" t="inlineStr"/>
+      <c r="R118" s="4" t="n"/>
       <c r="S118" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9659,7 +9676,7 @@
           <t>Hold + Pay after Hold</t>
         </is>
       </c>
-      <c r="R119" s="4" t="inlineStr"/>
+      <c r="R119" s="4" t="n"/>
       <c r="S119" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9730,7 +9747,7 @@
           <t>Hold + Pay after Hold</t>
         </is>
       </c>
-      <c r="R120" s="33" t="inlineStr"/>
+      <c r="R120" s="33" t="n"/>
       <c r="S120" s="33" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9803,7 +9820,7 @@
           <t>Not Bundle</t>
         </is>
       </c>
-      <c r="R121" s="4" t="inlineStr"/>
+      <c r="R121" s="4" t="n"/>
       <c r="S121" s="4" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -9876,10 +9893,10 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R122" s="4" t="inlineStr"/>
+      <c r="R122" s="4" t="n"/>
       <c r="S122" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9950,10 +9967,10 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R123" s="4" t="inlineStr"/>
+      <c r="R123" s="4" t="n"/>
       <c r="S123" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -10023,10 +10040,10 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R124" s="4" t="inlineStr"/>
+      <c r="R124" s="4" t="n"/>
       <c r="S124" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -10046,17 +10063,17 @@
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>Money still owed is reflected where the reports say it is</t>
+          <t>Extras bought with a booking are visible in the reports</t>
         </is>
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>An outstanding amount is not silently dropped.</t>
+          <t>The extras this supplier supports (seats, meals, bags or a fare package) are not lost between the booking and the reports.</t>
         </is>
       </c>
       <c r="F125" s="6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G125" s="4" t="inlineStr">
@@ -10066,14 +10083,15 @@
       </c>
       <c r="H125" s="4" t="inlineStr">
         <is>
-          <t>1. Note the 'Current Outstanding' figure shown with the wallet.
-2. Open the report that covers amounts due.
-3. Compare the two.</t>
+          <t>1. Check which extras the supplier supports (Seat, Meal, Baggage, Bundle) on its capability plan. Only those are in scope; do not look for the others.
+2. Make a booking that includes at least one of the supported extras.
+3. Note what you added and what each cost.
+4. Find that booking in the reports.</t>
         </is>
       </c>
       <c r="I125" s="4" t="inlineStr">
         <is>
-          <t>The report and the wallet tell the same story about what is owed. If nothing is owed, both say so. Neither shows an amount the other does not.</t>
+          <t>The amount the reports show for the booking includes what the supported extras cost, or the extras are listed in their own right. What was paid for is traceable - it does not vanish into a single figure that does not add up. If a report shows fare only by design, the difference is explained by the extras. Extras the supplier does not support are not expected and are not a failure.</t>
         </is>
       </c>
       <c r="J125" s="7" t="inlineStr">
@@ -10083,7 +10101,7 @@
       </c>
       <c r="K125" s="8" t="inlineStr">
         <is>
-          <t>Draft 28 Sep 2026 - written after the Statement report was found returning no data for a real paid booking (run-007). Deliberately generic: it applies to any supplier and any report, and names no fixed figures. Review = Pending: it does not run until approved.</t>
+          <t>Draft 28 Sep 2026 - written after the Statement report was found returning no data for a real paid booking (run-007). Deliberately generic: it applies to any supplier and any report, and names no fixed figures. Review = Pending: it does not run until approved. Updated 4 Oct 2026 (Mohanad Dawood): generic for any supplier - checks only the extras that supplier supports (Seat, Meal, Baggage, Bundle or any combination).</t>
         </is>
       </c>
       <c r="L125" s="3" t="n"/>
@@ -10096,164 +10114,18 @@
           <t>None</t>
         </is>
       </c>
-      <c r="R125" s="4" t="inlineStr"/>
+      <c r="R125" s="4" t="n"/>
       <c r="S125" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="150" customHeight="1">
-      <c r="A126" s="2" t="n">
-        <v>125</v>
-      </c>
-      <c r="B126" s="3" t="inlineStr">
-        <is>
-          <t>TC-RPT-005</t>
-        </is>
-      </c>
-      <c r="C126" s="4" t="inlineStr">
-        <is>
-          <t>X. Reports</t>
-        </is>
-      </c>
-      <c r="D126" s="5" t="inlineStr">
-        <is>
-          <t>A report with no results says so clearly and is not an error</t>
-        </is>
-      </c>
-      <c r="E126" s="4" t="inlineStr">
-        <is>
-          <t>An empty report is distinguishable from a broken one.</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G126" s="4" t="inlineStr">
-        <is>
-          <t>See the 'Before every test' sheet. A booking you have just made in this run, and the wallet balance noted before you made it.</t>
-        </is>
-      </c>
-      <c r="H126" s="4" t="inlineStr">
-        <is>
-          <t>1. Open any report.
-2. Search a date range you know has no activity (for example a range well in the past).
-3. Then search a range you know does have activity.</t>
-        </is>
-      </c>
-      <c r="I126" s="4" t="inlineStr">
-        <is>
-          <t>The empty search says plainly that there is nothing for that period, with the table headings still shown. The second search returns rows. An empty result for a period that definitely has activity is a defect - the report cannot be trusted to tell empty from broken.</t>
-        </is>
-      </c>
-      <c r="J126" s="7" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K126" s="8" t="inlineStr">
-        <is>
-          <t>Draft 28 Sep 2026 - written after the Statement report was found returning no data for a real paid booking (run-007). Deliberately generic: it applies to any supplier and any report, and names no fixed figures. Review = Pending: it does not run until approved.</t>
-        </is>
-      </c>
-      <c r="L126" s="3" t="n"/>
-      <c r="M126" s="4" t="n"/>
-      <c r="N126" s="4" t="n"/>
-      <c r="O126" s="4" t="n"/>
-      <c r="P126" s="4" t="n"/>
-      <c r="Q126" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="R126" s="4" t="inlineStr"/>
-      <c r="S126" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="150" customHeight="1">
-      <c r="A127" s="2" t="n">
-        <v>126</v>
-      </c>
-      <c r="B127" s="3" t="inlineStr">
-        <is>
-          <t>TC-RPT-006</t>
-        </is>
-      </c>
-      <c r="C127" s="4" t="inlineStr">
-        <is>
-          <t>X. Reports</t>
-        </is>
-      </c>
-      <c r="D127" s="5" t="inlineStr">
-        <is>
-          <t>Extras bought with a booking are visible in the reports</t>
-        </is>
-      </c>
-      <c r="E127" s="4" t="inlineStr">
-        <is>
-          <t>Seats, meals and bags are not lost between the booking and the reports.</t>
-        </is>
-      </c>
-      <c r="F127" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="G127" s="4" t="inlineStr">
-        <is>
-          <t>See the 'Before every test' sheet. A booking you have just made in this run, and the wallet balance noted before you made it.</t>
-        </is>
-      </c>
-      <c r="H127" s="4" t="inlineStr">
-        <is>
-          <t>1. Make a booking that includes at least one extra (a seat, a meal or a bag).
-2. Note what you added and what each cost.
-3. Find that booking in the reports.</t>
-        </is>
-      </c>
-      <c r="I127" s="4" t="inlineStr">
-        <is>
-          <t>The amount the reports show for the booking includes what the extras cost, or the extras are listed in their own right. What was paid for is traceable - it does not vanish into a single figure that does not add up. If a report shows fare only by design, the difference is explained by the extras.</t>
-        </is>
-      </c>
-      <c r="J127" s="7" t="inlineStr">
-        <is>
-          <t>Partly</t>
-        </is>
-      </c>
-      <c r="K127" s="8" t="inlineStr">
-        <is>
-          <t>Draft 28 Sep 2026 - written after the Statement report was found returning no data for a real paid booking (run-007). Deliberately generic: it applies to any supplier and any report, and names no fixed figures. Review = Pending: it does not run until approved.</t>
-        </is>
-      </c>
-      <c r="L127" s="3" t="n"/>
-      <c r="M127" s="4" t="n"/>
-      <c r="N127" s="4" t="n"/>
-      <c r="O127" s="4" t="n"/>
-      <c r="P127" s="4" t="n"/>
-      <c r="Q127" s="4" t="inlineStr">
-        <is>
-          <t>Seat + Meal + Baggage</t>
-        </is>
-      </c>
-      <c r="R127" s="4" t="inlineStr"/>
-      <c r="S127" s="4" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
+          <t>Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="150" customHeight="1"/>
+    <row r="127" ht="150" customHeight="1"/>
     <row r="128" ht="150" customHeight="1"/>
     <row r="129" ht="150" customHeight="1"/>
     <row r="130" ht="150" customHeight="1"/>
-    <row r="131" ht="150" customHeight="1"/>
-    <row r="132" ht="150" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:P80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10274,18 +10146,18 @@
     <col width="110" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Before every test - read this once</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="13" t="inlineStr"/>
-      <c r="B3" s="14" t="inlineStr"/>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+    <row r="3" ht="20.1" customHeight="1">
+      <c r="A3" s="13" t="n"/>
+      <c r="B3" s="14" t="n"/>
+    </row>
+    <row r="4" ht="39.95" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Where</t>
@@ -10297,7 +10169,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="39.95" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
           <t>Who</t>
@@ -10309,7 +10181,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1">
+    <row r="6" ht="39.95" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
           <t>What to search</t>
@@ -10321,7 +10193,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="39.95" customHeight="1">
       <c r="A7" s="15" t="inlineStr">
         <is>
           <t>NEVER press 'Book'</t>
@@ -10333,7 +10205,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
+    <row r="8" ht="39.95" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Two steps</t>
@@ -10345,19 +10217,19 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="13" t="inlineStr"/>
-      <c r="B9" s="14" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
+    <row r="9" ht="20.1" customHeight="1">
+      <c r="A9" s="13" t="n"/>
+      <c r="B9" s="14" t="n"/>
+    </row>
+    <row r="10" ht="20.1" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Words used in this sheet</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
+      <c r="B10" s="14" t="n"/>
+    </row>
+    <row r="11" ht="39.95" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
           <t>fare package (bundle)</t>
@@ -10369,7 +10241,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1">
+    <row r="12" ht="39.95" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>extras (ancillaries)</t>
@@ -10381,7 +10253,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1">
+    <row r="13" ht="39.95" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
           <t>left panel</t>
@@ -10393,7 +10265,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="40" customHeight="1">
+    <row r="14" ht="39.95" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>seat chart</t>
@@ -10405,7 +10277,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="40" customHeight="1">
+    <row r="15" ht="39.95" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
           <t>colour key</t>
@@ -10417,7 +10289,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1">
+    <row r="16" ht="39.95" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>section</t>
@@ -10429,7 +10301,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1">
+    <row r="17" ht="39.95" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
           <t>seats-chosen count</t>
@@ -10441,19 +10313,19 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="13" t="inlineStr"/>
-      <c r="B18" s="14" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
+    <row r="18" ht="20.1" customHeight="1">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="14" t="n"/>
+    </row>
+    <row r="19" ht="20.1" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Important rule for writing tests</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr"/>
-    </row>
-    <row r="20" ht="40" customHeight="1">
+      <c r="B19" s="14" t="n"/>
+    </row>
+    <row r="20" ht="39.95" customHeight="1">
       <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Never fix a row or seat number</t>
@@ -10465,7 +10337,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
+    <row r="21" ht="39.95" customHeight="1">
       <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Say which cabin and package</t>
@@ -10477,7 +10349,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="40" customHeight="1">
+    <row r="22" ht="39.95" customHeight="1">
       <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Staging warning</t>
@@ -10489,14 +10361,14 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="45" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Every booking run needs FRESH passenger names and document numbers.</t>
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="150" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
         <is>
           <t>The system refuses a second booking for a passenger whose name, date of birth and document already have one. It returns a clear message that is NEVER shown on screen, so the booking simply appears to do nothing. This is not a seat-map test - it is a constraint on how the tests are run.</t>
@@ -10517,19 +10389,17 @@
   <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="1" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Questions for the business</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="60" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Most questions were answered on 17 Sep 2026. Only the ones still open need a decision. An unanswered question does not stop a test running - run it, write down what happened, and do not mark it failed.</t>
@@ -10740,7 +10610,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Why a seat cannot be chosen - four reasons, two messages</t>
@@ -10826,7 +10696,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -10843,7 +10713,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t>By priority</t>
@@ -10911,7 +10781,7 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Can it be automated?</t>
@@ -10948,7 +10818,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
           <t>By group</t>

</xml_diff>